<commit_message>
final - primer producte
</commit_message>
<xml_diff>
--- a/seguiment_preus.xlsx
+++ b/seguiment_preus.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Integral" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Brut Nature 0.75cl" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Rosé 0.75cl" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,13 +29,22 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE8B8"/>
+        <bgColor rgb="00FFE8B8"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -56,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -150,7 +160,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Evolució de preu — Integral</a:t>
+              <a:t>Evolució de preu — Brut Nature 0.75cl</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -164,30 +174,30 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Integral'!A1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Integral'!$B$1:$D$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Integral'!$B$1:$D$1</f>
+              <f>'Brut Nature 0.75cl'!A1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
             </numRef>
           </val>
         </ser>
@@ -196,30 +206,1278 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Integral'!A2</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Integral'!$B$1:$D$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Integral'!$B$2:$D$2</f>
+              <f>'Brut Nature 0.75cl'!A2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$2</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A7</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A8</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="9"/>
+          <order val="9"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A10</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="11"/>
+          <order val="11"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="12"/>
+          <order val="12"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A13</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="13"/>
+          <order val="13"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="14"/>
+          <order val="14"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A15</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$15</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="15"/>
+          <order val="15"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A16</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$16</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="16"/>
+          <order val="16"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="17"/>
+          <order val="17"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A18</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="18"/>
+          <order val="18"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A19</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$19</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="19"/>
+          <order val="19"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="20"/>
+          <order val="20"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A21</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="21"/>
+          <order val="21"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$22</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="22"/>
+          <order val="22"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A23</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$23</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="23"/>
+          <order val="23"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A24</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$24</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="24"/>
+          <order val="24"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="25"/>
+          <order val="25"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A26</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="26"/>
+          <order val="26"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A27</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$27</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="27"/>
+          <order val="27"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A28</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="28"/>
+          <order val="28"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A29</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$29</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="29"/>
+          <order val="29"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A30</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$30</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="30"/>
+          <order val="30"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A31</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$31</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="31"/>
+          <order val="31"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A32</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$32</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="32"/>
+          <order val="32"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A33</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="33"/>
+          <order val="33"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A34</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$34</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="34"/>
+          <order val="34"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A35</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$35</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="35"/>
+          <order val="35"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A36</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$36</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="36"/>
+          <order val="36"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A37</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$37</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="37"/>
+          <order val="37"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A38</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$38</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="38"/>
+          <order val="38"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A39</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$39</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="39"/>
+          <order val="39"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A40</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="40"/>
+          <order val="40"/>
+          <tx>
+            <strRef>
+              <f>'Brut Nature 0.75cl'!A41</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Brut Nature 0.75cl'!$B$41</f>
             </numRef>
           </val>
         </ser>
@@ -333,12 +1591,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Rosé 0.75cl'!$B$1:$E$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Rosé 0.75cl'!$B$1:$E$1</f>
+              <f>'Rosé 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Rosé 0.75cl'!$B$1</f>
             </numRef>
           </val>
         </ser>
@@ -365,12 +1623,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Rosé 0.75cl'!$B$1:$E$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Rosé 0.75cl'!$B$2:$E$2</f>
+              <f>'Rosé 0.75cl'!$B$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Rosé 0.75cl'!$B$2</f>
             </numRef>
           </val>
         </ser>
@@ -443,7 +1701,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>3</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -470,7 +1728,7 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>3</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -782,7 +2040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -793,34 +2051,415 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>2026-06-29T00:23:47</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-29T00:23:54</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-29T18:55:30</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Ametller Origen</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>16.95</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bodeboca</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>16.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bodega Vidal</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>14.23</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BonArea</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>15.95</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bonpreu Esclat</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>15.69</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cal Angel</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>15.24</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cal Feru</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>16.65</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Caprabo</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>16.95</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Carviresa</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>15.48</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cash Montseny</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>14.05</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Celler de gelida</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>16.95</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Condis</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>16.95</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Decantalo</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>15.75</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Degusta'm</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Descorcha y bebe</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>17.95</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>EnBotella</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>15.48</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>EnterWine</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>15.197601</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Grau Online</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>15.68</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>La Branca</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>16.4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>La Fuente</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>17.45</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>La Vinateria</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Móntatelo en casa</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>18.91</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Private Celler</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>18.95</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Santa Cecilia</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>16.75</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Sorli</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>15.29</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TendaVins</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>16.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TotVi</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>15.8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Verema i Collita</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>15.9</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>Vinissimus</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>17.25</v>
-      </c>
-      <c r="C2" t="n">
-        <v>17.25</v>
-      </c>
-      <c r="D2" t="n">
-        <v>17.25</v>
+      <c r="B30" t="n">
+        <v>15.75</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Vino Premier</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>16.25</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>VinoVí</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Vinomada</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>16.25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Vinos  Online</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>16.11</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Vinos Baco</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>16.75</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Vinos Barcelona</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>15.9</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Vinos en Casa</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Vins Noe</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Vins a casa</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Vivónium</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>13.02</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Winepalace</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>16.85</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>🟧 Cel·les en taronja/cursiva = preu introduït manualment</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -835,7 +2474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -846,22 +2485,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>2026-06-29T00:21:47</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-29T00:22:05</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-29T00:23:08</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-29T00:24:12</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -874,14 +2498,12 @@
       <c r="B2" t="n">
         <v>17.65</v>
       </c>
-      <c r="C2" t="n">
-        <v>17.65</v>
-      </c>
-      <c r="D2" t="n">
-        <v>17.65</v>
-      </c>
-      <c r="E2" t="n">
-        <v>17.65</v>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>🟧 Cel·les en taronja/cursiva = preu introduït manualment</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>